<commit_message>
NPT App: Final industrial-ready version with dynamic colors, sticky navbar, mobile responsive, improved UI/UX
</commit_message>
<xml_diff>
--- a/filtered_npt.xlsx
+++ b/filtered_npt.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -463,7 +463,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2025-08-03 00:00:00</t>
+          <t>2025-07-05 00:00:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -473,20 +473,1161 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Mechanical</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Top drive</t>
+          <t>Mud handling system</t>
         </is>
       </c>
       <c r="E2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Observed S/shaker screens &amp; cutting trays fully choked with cuttings. Cleaned the same. </t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2025-07-06 00:00:00</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Repair</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Mechanical</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Mud pump</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>observed leakage from MP-2 piston. Rectified the same</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2025-07-06 00:00:00</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Repair</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Mechanical</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Top drive</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
         <v>1</v>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>While disconnecting TDS, obsd TDS rotation without command while running in Estimate mode and showing residual torque in Encoder mode. Tried rectification by electrical team but could not succeed. Decided to operate TDS in encoder mode. Ok</t>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Found leakage from W/Pipe. Arrested the same by tightening. Greased W/pipe.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2025-07-10 00:00:00</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Repair</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Mechanical</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Top drive</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Obsd TDS guide rollers (DS) out of track. Try to rectify the same couldn't rectified </t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2025-07-14 00:00:00</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Repair</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Mechanical</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Top drive</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>14</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Work on TDS as Rollers were out of track.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2025-07-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Repair</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Mechanical</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Top drive</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>18</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Drill Mech FSR worked on TDS to attend guide rollers fabrication and checked TDS track.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2025-07-16 00:00:00</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Repair</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Mechanical</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Top drive</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>24</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Drill Mech FSR worked on TDS. Fitted TDS Guide rollers. TDS track measurement &amp; correction by providing/removing shims IIP.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2025-07-17 00:00:00</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Repair</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Mechanical</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Top drive</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>24</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>TDS roller issue / INSPECTION OF TDS ROLLER GUIDE TRACKS</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2025-07-18 00:00:00</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Repair</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Mechanical</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Top drive</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>24</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>TDS roller issue / INSPECTION OF TDS ROLLER GUIDE TRACKS</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2025-07-19 00:00:00</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Repair</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Mechanical</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Top drive</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>18</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>TDS roller issue / INSPECTION OF TDS ROLLER GUIDE TRACKS</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2025-07-23 00:00:00</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Repair</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Mechanical</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Mud pump</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>5</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Obsd air lock at both MP1 &amp; MP3.Troubleshooting is going on</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2025-07-23 00:00:00</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Repair</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Mechanical</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Top drive</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>2</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Obsd hydraulic elevator unable to open due to “open denied” fault in no load condition.Rectified the same</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2025-07-23 00:00:00</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Repair</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Mechanical</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Top drive</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>TDS abnormal sound rectified by Drillmech Online Team</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2025-07-25 00:00:00</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Repair</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Mechanical</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Top drive</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Observed Leakage in Hydraulic Elevator. Rectified the same by Mech team</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2025-07-25 00:00:00</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Repair</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Mechanical</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Mud pump</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Observed leakage from D/Coupling of suction line MP-2.
+Rectified the same by mechanical team</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2025-07-25 00:00:00</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Repair</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Mechanical</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Mud pump</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Observed mud leakage from MP3 suction line dresser coupling, rectified the same by mechanical team</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2025-07-28 00:00:00</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Repair</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Mechanical</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Top drive</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>While reaming obsd elevator ODS arm detached from TDS link. Rectified the same by mechanical team</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2025-07-29 00:00:00</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Repair</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Mechanical</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Top drive</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>3</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>observed hydraulic hose of hydraulic elevator got damaged, replaced by team.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2025-07-29 00:00:00</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Repair</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Mechanical</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Tds/ hyd elevator</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Obsd hyd elevator not opening due to malfunctioning of load sensor. Rectified the same by mech team.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2025-07-29 00:00:00</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Repair</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Mechanical</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Tds/ hyd elevator</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Due to frequent issues in hyd elevator, removed hydraulic elevator connections by mech team, changed elevator links and R/up  manual elevato</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2025-07-30 00:00:00</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Repair</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Mechanical</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Tds/ hyd elevator</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Due to frequent issues in hyd elevator, removed hydraulic elevator connections by mech team, changed elevator links and R/up  manual elevato</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2025-08-18 00:00:00</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Repair</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Mechanical</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Top drive</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>FITTED TORSIONAL PLATES BETWEEN SAVER SUB &amp; L/IBOP.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2025-08-28 00:00:00</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Repair</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Mechanical</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Top drive</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>4</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>REMOVED NG-5 TDS CLAMP ASSEMBLY FROM THE TDS. REPAIRED HP2K1 TDS CLAMP ASSEMBLY PIN HOLE. FITTING OF THE SAME IIP.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2025-08-28 00:00:00</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Repair</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Mechanical</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Top drive</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>4</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>COMPLETED FITTING OF THE ASSEMBLY AND ITS HYDRAULIC CONNECTIONS. FUNCTION TESTED TDS CLAMP OK.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2025-09-10 00:00:00</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Repair</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Mechanical</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Top drive</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>CLEANED DRILL FLOOR AND TDS. M/A AND REMOVED ELEVATOR AND ELEVATOR LINKS OPEN PIPE HANDLER AND PRESSURE PLATES, REMOVED IBOP MECHANISM. CHANGING IBOP IIP</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2025-09-10 00:00:00</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Repair</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Mechanical</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Top drive</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>12</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>M/A FOR IBOP CHANGE AND B/OFF JOINT B/W UPPER IBOP AND FOSV. ALSO BREAK OFF JOINT B/W IBOP AND TDS SHAFT. NEW IBOP FITTED TO TDS AND TIGHTENED</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2025-09-10 00:00:00</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Repair</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Mechanical</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Top drive</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>2</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>FITTED ELEVATOR LINKS PRESSURE TESTED IBOP FOUND OK.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2025-09-10 00:00:00</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Repair</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Mechanical</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Mud pump</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>DURING C&amp;C @ C/SHOE ALL MPS FAULTED ELEC.TEAM RECTIFIED.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2025-09-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Repair</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Mechanical</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Top drive</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>12</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CONTD M/UP OF BHA, M/UP OF SAVER SUB AND X/OVER. WHILE M/UP OF STABILIZER WITH X/OVER FOUND TDS ROLLERS CAME OUT ITS TRACK.TRIED LOWERING TDS SLOWLEY </t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2025-09-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Repair</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Mechanical</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Top drive</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>2</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>OBSD TDS TILTED ONE SIDE AND H/UP ON THE TRACK FURTHER M/A TO LOWER TDS</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2025-09-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Repair</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Mechanical</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Top drive</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>4</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>REMOVED ROLLERS OF OUT-OF-TRACK TDS TRACK PLATES DS&amp; ODS *RRELESED LOAD ON THE PLATES</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2025-09-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Repair</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Mechanical</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Top drive</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>24</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>BROUGHT TDS DOWN TO DRILL FLOOR @SLOWSPEED IN FORMED AND HANDED OVER TDS TO ECHANICAL FOR PLATES AND ROLLERS INSPECTION CONTD. REMOVAL OF TDS ROLLER AND GUIDE PLATES. REMOVED REMAINING TWO GUIDE ROLLER ALONG PLATES &amp; GUIDE PLATE WITHOUT ROLLERS, WITH GREAT DIFFICULTY. OBSERVED TOTAL OF 07/16 ROLLERS DAMAGED.C/OUT HOUSEKEEPING AND CLEANING OF MAST AND DERRIC FLOOR. M/A AND DISCONNETED LINK TILT  AND REMOVED BOTH LINK</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2025-09-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Repair</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Mechanical</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Tds track</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>14</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>DRILL MECH FSR TEAM REPORTED AT SITE. CHECKED TDS TRACK GAP BETWEEN  SECTION 1-2 &amp; 2-3. FOUND LATERAL MISALIGNMENT BETWEEN SECTION 2-3. DECIDED TO REMOVE SHIMS AT START OF SECTION 3 AND  REMOVED  SHIMS AT START OF SECTION 3  &amp; ALIGNED 2ND &amp; 3RD SECTION</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2025-09-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Repair</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Mechanical</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Top drive</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>10</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FITTED 02 TDS GUIDE ROLLER PLATES </t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2025-09-14 00:00:00</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Repair</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Mechanical</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Top drive</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>24</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>TDS ROLLERS OUT OF TRACK INSPECTION BY DRILLMEC IIP</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2025-09-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Repair</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Mechanical</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Top drive</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>23</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>TDS ROLLERS OUT OF TRACK INSPECTION BY DRILLMEC IIP</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2025-09-16 00:00:00</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Repair</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Mechanical</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Top drive</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>12</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>RECTIFICATION OF TDS ROLLERS DONE MY MECHANICAL AND DRILLMEC TEAMS</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2025-10-19 00:00:00</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Repair</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Mechanical</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Top drive</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>1</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>OBSD PIPE GUIDE OF TD CLAMP ASSEMBLY STUCK TO S/SUB. RECTIFIED THE SAME. REPLACED D/PIPE</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2025-10-22 00:00:00</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Repair</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Mechanical</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Monkey board winch</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>3</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>MONKEY BOARD WINCH NOT WORKING. REPLACED THE SAME.</t>
         </is>
       </c>
     </row>

</xml_diff>